<commit_message>
Record DEF-002 as closed in the final records
Updates the PED, RTM, risk register, ADR-008 and README now that the audit trail's insert-only trigger has a direct test: NFR-007 is met and scope completion rises to 95.7% (44 of 46). The test count is 288 throughout.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v4.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v4.0.xlsx
@@ -524,7 +524,7 @@
     <row r="1" ht="17.25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CivicConnect Requirements Traceability Matrix (RTM) - v4.0 FINAL, release v1.0.0. Evidence: 287/287 automated tests pass (18 Oct 2026, PostgreSQL 17); simulated production 13/13 (Test/Evidence/Final_Simulated_Production.md). Columns W and X give each acceptance criterion's final status and each requirement's final outcome. Scope completion: 43.5 of 46 = 94.6% (PED v4.0).</t>
+          <t>CivicConnect Requirements Traceability Matrix (RTM) - v4.0 FINAL, release v1.0.0. Evidence: 288/288 automated tests pass (18 Oct 2026, PostgreSQL 17); simulated production 13/13 (Test/Evidence/Final_Simulated_Production.md). Columns W and X give each acceptance criterion's final status and each requirement's final outcome. Scope completion: 44 of 46 = 95.7% (PED v4.0).</t>
         </is>
       </c>
     </row>
@@ -4309,22 +4309,22 @@
       </c>
       <c r="U32" s="5" t="inlineStr">
         <is>
-          <t>HistoryInsertOnlyTests pass (automated, 16 Oct 2026): an UPDATE or DELETE on request_history is refused. The audit_entries trigger has no test of its own yet</t>
+          <t>HistoryInsertOnlyTests pass (automated, 18 Oct 2026): an UPDATE or DELETE on request_history or audit_entries is refused by the insert-only trigger (DEF-002 closed)</t>
         </is>
       </c>
       <c r="V32" s="5" t="inlineStr">
         <is>
-          <t>IN (CR-016); gap: no direct test of the audit_entries trigger</t>
+          <t>IN (CR-016)</t>
         </is>
       </c>
       <c r="W32" s="5" t="inlineStr">
         <is>
-          <t>Partially Met: history is insert-only and tested; the audit_entries trigger has no direct test (DEF-002)</t>
+          <t>Met: request_history and audit_entries are insert-only and both triggers are tested directly (DEF-002 closed)</t>
         </is>
       </c>
       <c r="X32" s="5" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>IMPLEMENTED (CR-016)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record the hosted release in the final records
Update the PED, RTM, risk register, README, ADRs, test plan and design docs for the live Render and Neon deployment, with NFR-001 and NFR-009 now Met (45 of 46, 97.8%). Add the hosted deployment check and fill in the CI evidence links.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v4.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v4.0.xlsx
@@ -524,7 +524,7 @@
     <row r="1" ht="17.25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CivicConnect Requirements Traceability Matrix (RTM) - v4.0 FINAL, release v1.0.0. Evidence: 288/288 automated tests pass (18 Oct 2026, PostgreSQL 17); simulated production 13/13 (Test/Evidence/Final_Simulated_Production.md). Columns W and X give each acceptance criterion's final status and each requirement's final outcome. Scope completion: 44 of 46 = 95.7% (PED v4.0).</t>
+          <t>CivicConnect Requirements Traceability Matrix (RTM) - v4.0 FINAL, release v1.0.0, live at https://sen381-project-group-i-2026.onrender.com/. Evidence: 288/288 automated tests pass (18 Oct 2026, PostgreSQL 17); simulated production 13/13 (Test/Evidence/Final_Simulated_Production.md); hosted checks (Test/Evidence/Hosted_Deployment_Check.md). Column O gives the M4 release evidence; columns W and X give each acceptance criterion's final status and each requirement's final outcome. Scope completion: 45 of 46 = 97.8% (PED v4.0).</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="55" customHeight="1">
+    <row r="3" ht="93.25" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>FR-001</t>
@@ -741,7 +741,7 @@
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
@@ -790,7 +790,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="55" customHeight="1">
+    <row r="4" ht="93.25" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>FR-002</t>
@@ -863,7 +863,7 @@
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42.25" customHeight="1">
+    <row r="5" ht="93.25" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>FR-003</t>
@@ -985,7 +985,7 @@
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P5" s="5" t="inlineStr">
@@ -1034,7 +1034,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42.25" customHeight="1">
+    <row r="6" ht="93.25" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>FR-004</t>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="O6" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
@@ -1156,7 +1156,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="42.25" customHeight="1">
+    <row r="7" ht="55" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>FR-005</t>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
         </is>
       </c>
       <c r="P7" s="5" t="inlineStr">
@@ -1336,22 +1336,22 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
+          <t>PR #34 (frontend-milestone-3-development, CR-016)</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
       <c r="O8" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
         </is>
       </c>
       <c r="P8" s="5" t="inlineStr">
@@ -1400,7 +1400,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="67.75" customHeight="1">
+    <row r="9" ht="93.25" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>FR-007</t>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P9" s="5" t="inlineStr">
@@ -1522,7 +1522,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42.25" customHeight="1">
+    <row r="10" ht="93.25" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>FR-008</t>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P10" s="5" t="inlineStr">
@@ -1644,7 +1644,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42.25" customHeight="1">
+    <row r="11" ht="93.25" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>FR-009</t>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P11" s="5" t="inlineStr">
@@ -1766,7 +1766,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="42.25" customHeight="1">
+    <row r="12" ht="93.25" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>FR-010</t>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="O12" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P12" s="5" t="inlineStr">
@@ -1888,7 +1888,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="67.75" customHeight="1">
+    <row r="13" ht="93.25" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>FR-011</t>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P13" s="5" t="inlineStr">
@@ -2010,7 +2010,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="80.5" customHeight="1">
+    <row r="14" ht="93.25" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>FR-012</t>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="O14" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr">
@@ -2132,7 +2132,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="38.25" customHeight="1">
+    <row r="15" ht="93.25" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>FR-013</t>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P15" s="5" t="inlineStr">
@@ -2254,7 +2254,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="42.25" customHeight="1">
+    <row r="16" ht="93.25" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>FR-014</t>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="O16" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); M3 acceptance checks pass (Test/Evidence/M3_Acceptance_Checks.md)</t>
         </is>
       </c>
       <c r="P16" s="5" t="inlineStr">
@@ -2434,22 +2434,22 @@
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
+          <t>PR #34 (frontend-milestone-3-development, CR-016)</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="N17" s="6" t="inlineStr">
         <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="N17" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
       <c r="O17" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
         </is>
       </c>
       <c r="P17" s="5" t="inlineStr">
@@ -2556,144 +2556,144 @@
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
+          <t>PR #34 (frontend-milestone-3-development, CR-016)</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Blocked pending CR-005</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="M18" s="5" t="inlineStr">
-        <is>
-          <t>Blocked pending CR-005</t>
-        </is>
-      </c>
-      <c r="N18" s="6" t="inlineStr">
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>Changed - blocked, CR-005 pending approval</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>M. Malope (CR); K. Marota (schema)</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Category.TargetResponseHours (default 72, set on Admin/Categories); Request.TargetResponseAtUtc fixed at submission (CR-005, migration AddRemainingRequirements); ResponseTarget.IsOverdue; Oversight Open and Overdue filter; overdue rows tagged on Oversight and Staff/Queue</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>ResponseTargetTests, CategoryServiceTests, SubmissionServiceTests (FR-016), ReportingTests (AC-016.1, AC-016.2, CR-005), StaffScreensTests (AC-016.2)</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>Open, resolved, closed and rejected requests are each identifiable; an open request past its target is flagged as overdue</t>
+        </is>
+      </c>
+      <c r="U18" s="5" t="inlineStr">
+        <is>
+          <t>ResponseTargetTests, CategoryServiceTests, SubmissionServiceTests, ReportingTests, StaffScreensTests pass (automated, 16 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="V18" s="5" t="inlineStr">
+        <is>
+          <t>IN (CR-016; CR-005 approved)</t>
+        </is>
+      </c>
+      <c r="W18" s="5" t="inlineStr">
+        <is>
+          <t>AC-016.1 Met; AC-016.2 Met</t>
+        </is>
+      </c>
+      <c r="X18" s="5" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED (CR-016; target field CR-005)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="55" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>FR-017</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>View request information by category/status (or another justified dimension).</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>ST-3</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>AC-017.1</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>ASR-04</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>FE oversight grouping -&gt; entry -&gt; Reporting -&gt; Requests API</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>No reporting copy; grouped through Requests</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>ADR-004; ADR-006</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>ADR-006</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>PR #34 (frontend-milestone-3-development, CR-016)</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
         <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="O18" s="6" t="inlineStr">
-        <is>
-          <t>at M4</t>
-        </is>
-      </c>
-      <c r="P18" s="5" t="inlineStr">
-        <is>
-          <t>Changed - blocked, CR-005 pending approval</t>
-        </is>
-      </c>
-      <c r="Q18" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope (CR); K. Marota (schema)</t>
-        </is>
-      </c>
-      <c r="R18" s="5" t="inlineStr">
-        <is>
-          <t>Category.TargetResponseHours (default 72, set on Admin/Categories); Request.TargetResponseAtUtc fixed at submission (CR-005, migration AddRemainingRequirements); ResponseTarget.IsOverdue; Oversight Open and Overdue filter; overdue rows tagged on Oversight and Staff/Queue</t>
-        </is>
-      </c>
-      <c r="S18" s="5" t="inlineStr">
-        <is>
-          <t>ResponseTargetTests, CategoryServiceTests, SubmissionServiceTests (FR-016), ReportingTests (AC-016.1, AC-016.2, CR-005), StaffScreensTests (AC-016.2)</t>
-        </is>
-      </c>
-      <c r="T18" s="5" t="inlineStr">
-        <is>
-          <t>Open, resolved, closed and rejected requests are each identifiable; an open request past its target is flagged as overdue</t>
-        </is>
-      </c>
-      <c r="U18" s="5" t="inlineStr">
-        <is>
-          <t>ResponseTargetTests, CategoryServiceTests, SubmissionServiceTests, ReportingTests, StaffScreensTests pass (automated, 16 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="V18" s="5" t="inlineStr">
-        <is>
-          <t>IN (CR-016; CR-005 approved)</t>
-        </is>
-      </c>
-      <c r="W18" s="5" t="inlineStr">
-        <is>
-          <t>AC-016.1 Met; AC-016.2 Met</t>
-        </is>
-      </c>
-      <c r="X18" s="5" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED (CR-016; target field CR-005)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="42.25" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>FR-017</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>View request information by category/status (or another justified dimension).</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>ST-3</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>AC-017.1</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>ASR-04</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>FE oversight grouping -&gt; entry -&gt; Reporting -&gt; Requests API</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>No reporting copy; grouped through Requests</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>ADR-004; ADR-006</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>ADR-006</t>
-        </is>
-      </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="N19" s="6" t="inlineStr">
         <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
-      <c r="N19" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
       <c r="O19" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
         </is>
       </c>
       <c r="P19" s="5" t="inlineStr">
@@ -2800,22 +2800,22 @@
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
+          <t>PR #34 (frontend-milestone-3-development, CR-016)</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="M20" s="6" t="inlineStr">
+      <c r="N20" s="6" t="inlineStr">
         <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="N20" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
       <c r="O20" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
         </is>
       </c>
       <c r="P20" s="5" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); simulated production 13/13 with real sign-in</t>
         </is>
       </c>
       <c r="P21" s="5" t="inlineStr">
@@ -2986,7 +2986,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="55" customHeight="1">
+    <row r="22" ht="80.5" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>FR-020</t>
@@ -3059,7 +3059,7 @@
       </c>
       <c r="O22" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); simulated production 13/13 with real sign-in</t>
         </is>
       </c>
       <c r="P22" s="5" t="inlineStr">
@@ -3108,7 +3108,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="42.25" customHeight="1">
+    <row r="23" ht="55" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>FR-021</t>
@@ -3166,400 +3166,400 @@
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
+          <t>PR #34 (frontend-milestone-3-development, CR-016)</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>Category table supports retire; no admin screen</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="M23" s="6" t="inlineStr">
-        <is>
-          <t>Category table supports retire; no admin screen</t>
-        </is>
-      </c>
-      <c r="N23" s="6" t="inlineStr">
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>Baselined</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>G. Enright with M. Malope</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>CategoryService (add, rename, retire, restore, set target); Admin/Categories; the submit form reads the live list</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>CategoryServiceTests (FR-021), ManagementScreensTests (FR-021)</t>
+        </is>
+      </c>
+      <c r="T23" s="5" t="inlineStr">
+        <is>
+          <t>An administrator changes the category list with no code change and the submit form follows; duplicate names refused</t>
+        </is>
+      </c>
+      <c r="U23" s="5" t="inlineStr">
+        <is>
+          <t>CategoryServiceTests, ManagementScreensTests pass (automated, 16 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="V23" s="5" t="inlineStr">
+        <is>
+          <t>IN (CR-016)</t>
+        </is>
+      </c>
+      <c r="W23" s="5" t="inlineStr">
+        <is>
+          <t>AC-021.1 Met</t>
+        </is>
+      </c>
+      <c r="X23" s="5" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED (CR-016)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="55" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>FR-022</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Access an audit trail of key controlled actions.</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>ST-4</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>AC-022.1</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>ASR-03</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>FE admin audit -&gt; entry -&gt; Requests history, plus Access and ReferenceData change records</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Append-only history in each owning schema</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>ADR-002 append-only; ADR-005 read permission</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>ADR-002; NFR-007; RSK-013</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>Backend branch</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>request_status_history and request_note with block_history_changes triggers. Admin view not built</t>
+        </is>
+      </c>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>Not in CI: Backend RealDatabaseTests (History_rows_cannot_be_changed_or_deleted). Planned in CI</t>
+        </is>
+      </c>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>Changed (CR-010)</t>
+        </is>
+      </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>G. Enright with K. Marota</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>Admin/Audit combines request history with the insert-only audit_entries table (category, user and role changes), filtered by kind</t>
+        </is>
+      </c>
+      <c r="S24" s="5" t="inlineStr">
+        <is>
+          <t>ManagementScreensTests (FR-022), UserAdminTests (FR-022), AttachmentTests</t>
+        </is>
+      </c>
+      <c r="T24" s="5" t="inlineStr">
+        <is>
+          <t>Key controlled actions are listed with actor and time, for administrators only</t>
+        </is>
+      </c>
+      <c r="U24" s="5" t="inlineStr">
+        <is>
+          <t>ManagementScreensTests, UserAdminTests, AttachmentTests pass (automated, 16 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="V24" s="5" t="inlineStr">
+        <is>
+          <t>IN (CR-016)</t>
+        </is>
+      </c>
+      <c r="W24" s="5" t="inlineStr">
+        <is>
+          <t>AC-022.1 Met</t>
+        </is>
+      </c>
+      <c r="X24" s="5" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED (CR-016)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="55" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>FR-023</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Access high-level service-performance and accountability reporting.</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>ST-5</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>AC-023.1</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>ASR-04</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>FE summary reports -&gt; entry -&gt; Reporting -&gt; Requests API</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Same figures as FR-018 at summary scope</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>ADR-004</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>CR-007; RSK-018</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>PR #34 (frontend-milestone-3-development, CR-016)</t>
+        </is>
+      </c>
+      <c r="M25" s="6" t="inlineStr">
         <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="O23" s="6" t="inlineStr">
-        <is>
-          <t>at M4</t>
-        </is>
-      </c>
-      <c r="P23" s="5" t="inlineStr">
-        <is>
-          <t>Baselined</t>
-        </is>
-      </c>
-      <c r="Q23" s="5" t="inlineStr">
-        <is>
-          <t>G. Enright with M. Malope</t>
-        </is>
-      </c>
-      <c r="R23" s="5" t="inlineStr">
-        <is>
-          <t>CategoryService (add, rename, retire, restore, set target); Admin/Categories; the submit form reads the live list</t>
-        </is>
-      </c>
-      <c r="S23" s="5" t="inlineStr">
-        <is>
-          <t>CategoryServiceTests (FR-021), ManagementScreensTests (FR-021)</t>
-        </is>
-      </c>
-      <c r="T23" s="5" t="inlineStr">
-        <is>
-          <t>An administrator changes the category list with no code change and the submit form follows; duplicate names refused</t>
-        </is>
-      </c>
-      <c r="U23" s="5" t="inlineStr">
-        <is>
-          <t>CategoryServiceTests, ManagementScreensTests pass (automated, 16 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="V23" s="5" t="inlineStr">
-        <is>
-          <t>IN (CR-016)</t>
-        </is>
-      </c>
-      <c r="W23" s="5" t="inlineStr">
-        <is>
-          <t>AC-021.1 Met</t>
-        </is>
-      </c>
-      <c r="X23" s="5" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED (CR-016)</t>
+      <c r="N25" s="6" t="inlineStr">
+        <is>
+          <t>at M3</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>Baselined - access model pending CR-007</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>M. Malope</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Sponsor role (CR-007); Pages/Reports/Summary reuses the oversight figures at summary level, with no individual requests</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>ReportingTests (AC-023.1), RequestAccessTests (FR-023)</t>
+        </is>
+      </c>
+      <c r="T25" s="5" t="inlineStr">
+        <is>
+          <t>Sponsors, managers and administrators see summary figures that match the records; sponsors see no request details</t>
+        </is>
+      </c>
+      <c r="U25" s="5" t="inlineStr">
+        <is>
+          <t>ReportingTests, RequestAccessTests pass (automated, 16 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="V25" s="5" t="inlineStr">
+        <is>
+          <t>IN (CR-016; CR-007 approved)</t>
+        </is>
+      </c>
+      <c r="W25" s="5" t="inlineStr">
+        <is>
+          <t>AC-023.1 Met</t>
+        </is>
+      </c>
+      <c r="X25" s="5" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED (CR-016; sponsor view CR-007)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="42.25" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>FR-022</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Access an audit trail of key controlled actions.</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>ST-4</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
+    <row r="26" ht="67.75" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>NFR-001</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Usability: a first-time requester can submit in ≤ 5 steps / 5 min.</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>ST-1</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>AC-022.1</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>ASR-03</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>FE admin audit -&gt; entry -&gt; Requests history, plus Access and ReferenceData change records</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Append-only history in each owning schema</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>ADR-002 append-only; ADR-005 read permission</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>ADR-002; NFR-007; RSK-013</t>
-        </is>
-      </c>
-      <c r="L24" s="6" t="inlineStr">
-        <is>
-          <t>Backend branch</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="inlineStr">
-        <is>
-          <t>request_status_history and request_note with block_history_changes triggers. Admin view not built</t>
-        </is>
-      </c>
-      <c r="N24" s="6" t="inlineStr">
-        <is>
-          <t>Not in CI: Backend RealDatabaseTests (History_rows_cannot_be_changed_or_deleted). Planned in CI</t>
-        </is>
-      </c>
-      <c r="O24" s="6" t="inlineStr">
-        <is>
-          <t>at M4</t>
-        </is>
-      </c>
-      <c r="P24" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>≤ 5 steps and ≤ 5 min (usability test)</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>ASR-06</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>FE guided submit form</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>ADR-004 one guided flow with per-field validation</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>ADR-004; RSK-016</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>UI branch</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>One guided form on Pages/Requests/Submit.cshtml with a message against each field</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Planned: moderated walkthrough with three first time users</t>
+        </is>
+      </c>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>v1.0.0: timed first-user walkthrough met the target (PED v4.0, M1 Scope to Final Delivery)</t>
+        </is>
+      </c>
+      <c r="P26" s="5" t="inlineStr">
         <is>
           <t>Changed (CR-010)</t>
         </is>
       </c>
-      <c r="Q24" s="5" t="inlineStr">
-        <is>
-          <t>G. Enright with K. Marota</t>
-        </is>
-      </c>
-      <c r="R24" s="5" t="inlineStr">
-        <is>
-          <t>Admin/Audit combines request history with the insert-only audit_entries table (category, user and role changes), filtered by kind</t>
-        </is>
-      </c>
-      <c r="S24" s="5" t="inlineStr">
-        <is>
-          <t>ManagementScreensTests (FR-022), UserAdminTests (FR-022), AttachmentTests</t>
-        </is>
-      </c>
-      <c r="T24" s="5" t="inlineStr">
-        <is>
-          <t>Key controlled actions are listed with actor and time, for administrators only</t>
-        </is>
-      </c>
-      <c r="U24" s="5" t="inlineStr">
-        <is>
-          <t>ManagementScreensTests, UserAdminTests, AttachmentTests pass (automated, 16 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="V24" s="5" t="inlineStr">
-        <is>
-          <t>IN (CR-016)</t>
-        </is>
-      </c>
-      <c r="W24" s="5" t="inlineStr">
-        <is>
-          <t>AC-022.1 Met</t>
-        </is>
-      </c>
-      <c r="X24" s="5" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED (CR-016)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="42.25" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>FR-023</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Access high-level service-performance and accountability reporting.</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>ST-5</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>AC-023.1</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>ASR-04</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>FE summary reports -&gt; entry -&gt; Reporting -&gt; Requests API</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Same figures as FR-018 at summary scope</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>ADR-004</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>CR-007; RSK-018</t>
-        </is>
-      </c>
-      <c r="L25" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
-      <c r="M25" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
-      <c r="N25" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
-      <c r="O25" s="6" t="inlineStr">
-        <is>
-          <t>at M4</t>
-        </is>
-      </c>
-      <c r="P25" s="5" t="inlineStr">
-        <is>
-          <t>Baselined - access model pending CR-007</t>
-        </is>
-      </c>
-      <c r="Q25" s="5" t="inlineStr">
+      <c r="Q26" s="5" t="inlineStr">
         <is>
           <t>M. Malope</t>
         </is>
       </c>
-      <c r="R25" s="5" t="inlineStr">
-        <is>
-          <t>Sponsor role (CR-007); Pages/Reports/Summary reuses the oversight figures at summary level, with no individual requests</t>
-        </is>
-      </c>
-      <c r="S25" s="5" t="inlineStr">
-        <is>
-          <t>ReportingTests (AC-023.1), RequestAccessTests (FR-023)</t>
-        </is>
-      </c>
-      <c r="T25" s="5" t="inlineStr">
-        <is>
-          <t>Sponsors, managers and administrators see summary figures that match the records; sponsors see no request details</t>
-        </is>
-      </c>
-      <c r="U25" s="5" t="inlineStr">
-        <is>
-          <t>ReportingTests, RequestAccessTests pass (automated, 16 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="V25" s="5" t="inlineStr">
-        <is>
-          <t>IN (CR-016; CR-007 approved)</t>
-        </is>
-      </c>
-      <c r="W25" s="5" t="inlineStr">
-        <is>
-          <t>AC-023.1 Met</t>
-        </is>
-      </c>
-      <c r="X25" s="5" t="inlineStr">
-        <is>
-          <t>IMPLEMENTED (CR-016; sponsor view CR-007)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="29.5" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>NFR-001</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Usability: a first-time requester can submit in ≤ 5 steps / 5 min.</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>ST-1</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>≤ 5 steps and ≤ 5 min (usability test)</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>ASR-06</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>FE guided submit form</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>ADR-004 one guided flow with per-field validation</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
-        </is>
-      </c>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>ADR-004; RSK-016</t>
-        </is>
-      </c>
-      <c r="L26" s="5" t="inlineStr">
-        <is>
-          <t>UI branch</t>
-        </is>
-      </c>
-      <c r="M26" s="5" t="inlineStr">
-        <is>
-          <t>One guided form on Pages/Requests/Submit.cshtml with a message against each field</t>
-        </is>
-      </c>
-      <c r="N26" s="5" t="inlineStr">
-        <is>
-          <t>Planned: moderated walkthrough with three first time users</t>
-        </is>
-      </c>
-      <c r="O26" s="6" t="inlineStr">
-        <is>
-          <t>at M4</t>
-        </is>
-      </c>
-      <c r="P26" s="5" t="inlineStr">
-        <is>
-          <t>Changed (CR-010)</t>
-        </is>
-      </c>
-      <c r="Q26" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope</t>
-        </is>
-      </c>
       <c r="R26" s="5" t="inlineStr">
         <is>
           <t>Pages/Requests/Submit: title, description, location, category, submit (five steps)</t>
@@ -3577,22 +3577,22 @@
       </c>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>Walkthrough not run: needs a timed first-time user</t>
+          <t>Timed first-user walkthrough run: met the five-step, five-minute target (PED v4.0, M1 Scope to Final Delivery)</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
         <is>
-          <t>IN*: walkthrough pending (Role 1)</t>
+          <t>IN: walkthrough done (Role 1)</t>
         </is>
       </c>
       <c r="W26" s="5" t="inlineStr">
         <is>
-          <t>Partially Met: the five-step form is built; the timed first-user walkthrough has not been run</t>
+          <t>Met: a first-time requester submitted without training within 5 steps and 5 minutes</t>
         </is>
       </c>
       <c r="X26" s="5" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED</t>
+          <t>IMPLEMENTED</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
         </is>
       </c>
       <c r="P27" s="5" t="inlineStr">
@@ -3718,7 +3718,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="42.25" customHeight="1">
+    <row r="28" ht="55" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>NFR-003</t>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="O28" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr">
@@ -3840,7 +3840,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="42.25" customHeight="1">
+    <row r="29" ht="93.25" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
           <t>NFR-004</t>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: PT-01 p95 0.064 s (Test/Evidence/PT-01_Results.md); hosted pages p95 under 1 s (Test/Evidence/Hosted_Deployment_Check.md)</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="W29" s="5" t="inlineStr">
         <is>
-          <t>Met locally: PT-01 p95 0.064 s against 3 s; not measured on a hosted server</t>
+          <t>Met: PT-01 p95 0.064 s locally against 3 s at 1,000 requests; on the hosted site the public pages answer with a p95 under 1 s (the queue itself was not timed there)</t>
         </is>
       </c>
       <c r="X29" s="5" t="inlineStr">
@@ -3962,7 +3962,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="38.25" customHeight="1">
+    <row r="30" ht="55" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>NFR-005</t>
@@ -4035,7 +4035,7 @@
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
         </is>
       </c>
       <c r="P30" s="5" t="inlineStr">
@@ -4084,7 +4084,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="55" customHeight="1">
+    <row r="31" ht="131.5" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
           <t>NFR-006</t>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="O31" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026); simulated production 13/13 with real sign-in; the live site refuses anonymous access (Test/Evidence/Hosted_Deployment_Check.md)</t>
         </is>
       </c>
       <c r="P31" s="5" t="inlineStr">
@@ -4206,7 +4206,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="55" customHeight="1">
+    <row r="32" ht="93.25" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>NFR-007</t>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026), including the DEF-002 test (HistoryInsertOnlyTests)</t>
         </is>
       </c>
       <c r="P32" s="5" t="inlineStr">
@@ -4328,7 +4328,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="42.25" customHeight="1">
+    <row r="33" ht="55" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
           <t>NFR-008</t>
@@ -4386,22 +4386,22 @@
       </c>
       <c r="L33" s="6" t="inlineStr">
         <is>
+          <t>PR #34 (frontend-milestone-3-development, CR-016)</t>
+        </is>
+      </c>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>Reporting reads the same tables; no reporting screen yet</t>
+        </is>
+      </c>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="M33" s="6" t="inlineStr">
-        <is>
-          <t>Reporting reads the same tables; no reporting screen yet</t>
-        </is>
-      </c>
-      <c r="N33" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
       <c r="O33" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: the column U tests pass (288/288, CI green on main, 18/10/2026)</t>
         </is>
       </c>
       <c r="P33" s="5" t="inlineStr">
@@ -4450,7 +4450,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="42.25" customHeight="1">
+    <row r="34" ht="80.5" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>NFR-009</t>
@@ -4508,12 +4508,12 @@
       </c>
       <c r="L34" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>PR #39 (Host setup: Dockerfile and Render deployment)</t>
         </is>
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>Not deployed yet; plan limits recorded in ADR-007</t>
+          <t>Deployed: Dockerfile on a Render Free web service, database on Neon Free (PR #39); plan limits in ADR-007</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="O34" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>v1.0.0: live on Render Free and Neon Free at $0 per month (Test/Evidence/Hosted_Deployment_Check.md; ADR-007)</t>
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr">
@@ -4563,16 +4563,16 @@
       </c>
       <c r="W34" s="5" t="inlineStr">
         <is>
-          <t>Partially Met: $0 plan documented (ADR-007) and runs with no paid service in simulated production; not proven on a hosted free tier</t>
+          <t>Met: runs live on Render Free and Neon Free at $0 per month (both plans confirmed Free); cost and limits recorded in ADR-007</t>
         </is>
       </c>
       <c r="X34" s="5" t="inlineStr">
         <is>
-          <t>PARTIALLY IMPLEMENTED (TD-04)</t>
+          <t>IMPLEMENTED (TD-04 repaid)</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="29.5" customHeight="1">
+    <row r="35" ht="55" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
           <t>NFR-010</t>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="L35" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>None: the service split was not built (CR-014)</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
-          <t>at M4</t>
+          <t>None: not implemented; accepted as technical debt (CR-014, TD-01)</t>
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr">

</xml_diff>